<commit_message>
pk filtering removed, clean output involved
</commit_message>
<xml_diff>
--- a/excel_files/analytics_dw.public.dim_vehicle_master.xlsx
+++ b/excel_files/analytics_dw.public.dim_vehicle_master.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PycharmProjects\ETL_Testing_Databricks_Multi_Source\Extract\excel_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PycharmProjects\ETL_Testing_Databricks_Multi_Source\Execution\excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56809F17-F322-446A-9B00-9F39EC242071}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E115370A-859D-4C2E-8CC3-1F262005D3D6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6936" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,12 +18,12 @@
     <sheet name="_joins" sheetId="2" r:id="rId3"/>
     <sheet name="_parameters" sheetId="3" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="195">
   <si>
     <t>SOURCE</t>
   </si>
@@ -508,118 +508,106 @@
     <t>SUB_PATH</t>
   </si>
   <si>
+    <t>Sub-path inside blob storage (e.g. xl)</t>
+  </si>
+  <si>
+    <t>STORAGE_ACCOUNT</t>
+  </si>
+  <si>
+    <t>Azure storage account name (e.g. etlstorage0907)</t>
+  </si>
+  <si>
+    <t>CONTAINER</t>
+  </si>
+  <si>
+    <t>Azure blob container name (e.g. etl-source-data)</t>
+  </si>
+  <si>
+    <t>VERIFY_SCHEMA</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>Run Snowflake schema verification: true / false</t>
+  </si>
+  <si>
+    <t>full</t>
+  </si>
+  <si>
+    <t>DATE_WATERMARK_MODE</t>
+  </si>
+  <si>
+    <t>Date watermark mode: full / range</t>
+  </si>
+  <si>
+    <t>DATE_FROM</t>
+  </si>
+  <si>
+    <t>(Optional) Date watermark start  YYYY-MM-DD</t>
+  </si>
+  <si>
+    <t>DATE_FROM_COL</t>
+  </si>
+  <si>
+    <t>(Optional) Column name for DATE_FROM filter</t>
+  </si>
+  <si>
+    <t>DATE_TO</t>
+  </si>
+  <si>
+    <t>(Optional) Date watermark end    YYYY-MM-DD</t>
+  </si>
+  <si>
+    <t>DATE_TO_COL</t>
+  </si>
+  <si>
+    <t>(Optional) Column name for DATE_TO filter</t>
+  </si>
+  <si>
+    <t>PARTIAL_COLS</t>
+  </si>
+  <si>
+    <t>(Optional) Comma-separated target column names for partial run</t>
+  </si>
+  <si>
+    <t>RUN_SYNTAX_CHECK</t>
+  </si>
+  <si>
+    <t>Run Excel syntax check before parsing: true / false</t>
+  </si>
+  <si>
+    <t>EXCEL_FILE</t>
+  </si>
+  <si>
+    <t>analytics_dw.public.dim_vehicle_master.xlsx</t>
+  </si>
+  <si>
+    <t>This Excel file name (e.g. analytics_dw.public.dim_vehicle_master.xlsx)</t>
+  </si>
+  <si>
+    <t>SF_DATABASE</t>
+  </si>
+  <si>
+    <t>(Optional) Snowflake database override (e.g. ANALYTICS_DW)</t>
+  </si>
+  <si>
+    <t>dbo</t>
+  </si>
+  <si>
+    <t>CLEAN_OUTPUT</t>
+  </si>
+  <si>
+    <t>This togle will delete the old runbook folder for table at each run</t>
+  </si>
+  <si>
+    <t>etl_output_mysql_xl_p</t>
+  </si>
+  <si>
+    <t>etl_output_server_xl_p</t>
+  </si>
+  <si>
     <t>xl</t>
-  </si>
-  <si>
-    <t>Sub-path inside blob storage (e.g. xl)</t>
-  </si>
-  <si>
-    <t>STORAGE_ACCOUNT</t>
-  </si>
-  <si>
-    <t>Azure storage account name (e.g. etlstorage0907)</t>
-  </si>
-  <si>
-    <t>CONTAINER</t>
-  </si>
-  <si>
-    <t>Azure blob container name (e.g. etl-source-data)</t>
-  </si>
-  <si>
-    <t>VERIFY_SCHEMA</t>
-  </si>
-  <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>Run Snowflake schema verification: true / false</t>
-  </si>
-  <si>
-    <t>PK_FILTER_MODE</t>
-  </si>
-  <si>
-    <t>full</t>
-  </si>
-  <si>
-    <t>PK filter mode: full / range / set</t>
-  </si>
-  <si>
-    <t>DATE_WATERMARK_MODE</t>
-  </si>
-  <si>
-    <t>Date watermark mode: full / range</t>
-  </si>
-  <si>
-    <t>PK_RANGE_LOWER</t>
-  </si>
-  <si>
-    <t>(Optional) PK range lower bound integer</t>
-  </si>
-  <si>
-    <t>PK_RANGE_UPPER</t>
-  </si>
-  <si>
-    <t>(Optional) PK range upper bound integer</t>
-  </si>
-  <si>
-    <t>DATE_FROM</t>
-  </si>
-  <si>
-    <t>(Optional) Date watermark start  YYYY-MM-DD</t>
-  </si>
-  <si>
-    <t>DATE_FROM_COL</t>
-  </si>
-  <si>
-    <t>(Optional) Column name for DATE_FROM filter</t>
-  </si>
-  <si>
-    <t>DATE_TO</t>
-  </si>
-  <si>
-    <t>(Optional) Date watermark end    YYYY-MM-DD</t>
-  </si>
-  <si>
-    <t>DATE_TO_COL</t>
-  </si>
-  <si>
-    <t>(Optional) Column name for DATE_TO filter</t>
-  </si>
-  <si>
-    <t>PARTIAL_COLS</t>
-  </si>
-  <si>
-    <t>(Optional) Comma-separated target column names for partial run</t>
-  </si>
-  <si>
-    <t>RUN_SYNTAX_CHECK</t>
-  </si>
-  <si>
-    <t>Run Excel syntax check before parsing: true / false</t>
-  </si>
-  <si>
-    <t>EXCEL_FILE</t>
-  </si>
-  <si>
-    <t>analytics_dw.public.dim_vehicle_master.xlsx</t>
-  </si>
-  <si>
-    <t>This Excel file name (e.g. analytics_dw.public.dim_vehicle_master.xlsx)</t>
-  </si>
-  <si>
-    <t>SF_DATABASE</t>
-  </si>
-  <si>
-    <t>(Optional) Snowflake database override (e.g. ANALYTICS_DW)</t>
-  </si>
-  <si>
-    <t>dbo</t>
-  </si>
-  <si>
-    <t>etl_output_server_xl_p</t>
-  </si>
-  <si>
-    <t>etl_output_mysql_xl_p</t>
   </si>
 </sst>
 </file>
@@ -668,7 +656,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -718,6 +706,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -787,7 +787,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -818,6 +818,18 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1159,32 +1171,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="18" t="s">
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="16"/>
-      <c r="K1" s="14" t="s">
+      <c r="J1" s="20"/>
+      <c r="K1" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="15"/>
-      <c r="O1" s="16"/>
-      <c r="P1" s="17" t="s">
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="15"/>
-      <c r="R1" s="16"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="20"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -1244,7 +1256,7 @@
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5" t="s">
@@ -1292,7 +1304,7 @@
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6" t="s">
@@ -1332,7 +1344,7 @@
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5" t="s">
@@ -1372,7 +1384,7 @@
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6" t="s">
@@ -1412,7 +1424,7 @@
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="5" t="s">
@@ -1454,7 +1466,7 @@
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6" t="s">
@@ -1494,7 +1506,7 @@
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="5" t="s">
@@ -1534,7 +1546,7 @@
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6" t="s">
@@ -1578,7 +1590,7 @@
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5" t="s">
@@ -1618,7 +1630,7 @@
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6" t="s">
@@ -1658,7 +1670,7 @@
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5" t="s">
@@ -1706,7 +1718,7 @@
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6" t="s">
@@ -1752,7 +1764,7 @@
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5" t="s">
@@ -1792,7 +1804,7 @@
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6" t="s">
@@ -1832,7 +1844,7 @@
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5" t="s">
@@ -1874,7 +1886,7 @@
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6" t="s">
@@ -1916,7 +1928,7 @@
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5" t="s">
@@ -1964,7 +1976,7 @@
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6" t="s">
@@ -2010,7 +2022,7 @@
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5" t="s">
@@ -2050,7 +2062,7 @@
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="6" t="s">
@@ -2094,7 +2106,7 @@
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5" t="s">
@@ -2134,7 +2146,7 @@
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6" t="s">
@@ -2182,7 +2194,7 @@
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B25" s="5"/>
       <c r="C25" s="5" t="s">
@@ -2228,7 +2240,7 @@
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6" t="s">
@@ -2272,7 +2284,7 @@
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5" t="s">
@@ -2312,7 +2324,7 @@
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="6" t="s">
@@ -2535,32 +2547,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="18" t="s">
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="16"/>
-      <c r="K1" s="14" t="s">
+      <c r="J1" s="20"/>
+      <c r="K1" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="15"/>
-      <c r="O1" s="16"/>
-      <c r="P1" s="17" t="s">
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="15"/>
-      <c r="R1" s="16"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="20"/>
     </row>
     <row r="2" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -2620,10 +2632,10 @@
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>22</v>
@@ -2670,10 +2682,10 @@
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>22</v>
@@ -2712,10 +2724,10 @@
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>22</v>
@@ -2754,10 +2766,10 @@
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>22</v>
@@ -2796,10 +2808,10 @@
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>22</v>
@@ -2840,10 +2852,10 @@
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>22</v>
@@ -2882,10 +2894,10 @@
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>22</v>
@@ -2924,10 +2936,10 @@
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>22</v>
@@ -2970,10 +2982,10 @@
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>22</v>
@@ -3012,10 +3024,10 @@
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>22</v>
@@ -3054,10 +3066,10 @@
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>22</v>
@@ -3104,10 +3116,10 @@
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>71</v>
@@ -3152,10 +3164,10 @@
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>71</v>
@@ -3194,10 +3206,10 @@
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>71</v>
@@ -3236,10 +3248,10 @@
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>71</v>
@@ -3280,10 +3292,10 @@
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>71</v>
@@ -3324,10 +3336,10 @@
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>71</v>
@@ -3374,10 +3386,10 @@
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>88</v>
@@ -3422,10 +3434,10 @@
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>88</v>
@@ -3464,10 +3476,10 @@
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>88</v>
@@ -3510,10 +3522,10 @@
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>88</v>
@@ -3552,10 +3564,10 @@
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>88</v>
@@ -3602,10 +3614,10 @@
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>104</v>
@@ -3650,10 +3662,10 @@
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>104</v>
@@ -3696,10 +3708,10 @@
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>104</v>
@@ -3738,10 +3750,10 @@
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C28" s="6" t="s">
         <v>104</v>
@@ -4015,7 +4027,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -4060,10 +4072,10 @@
         <v>160</v>
       </c>
       <c r="C3" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="D3" s="13" t="s">
         <v>161</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -4071,11 +4083,11 @@
         <v>3</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C4" s="10"/>
       <c r="D4" s="11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -4083,11 +4095,11 @@
         <v>4</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -4095,112 +4107,114 @@
         <v>5</v>
       </c>
       <c r="B6" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="D6" s="11" t="s">
         <v>168</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>6</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D7" s="15" t="s">
         <v>171</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="10">
         <v>7</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="16" t="s">
+        <v>172</v>
+      </c>
+      <c r="C8" s="16"/>
+      <c r="D8" s="17" t="s">
         <v>173</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>171</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="12">
         <v>8</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C9" s="14"/>
+      <c r="D9" s="15" t="s">
         <v>175</v>
-      </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="13" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="10">
         <v>9</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="16" t="s">
+        <v>176</v>
+      </c>
+      <c r="C10" s="16"/>
+      <c r="D10" s="17" t="s">
         <v>177</v>
-      </c>
-      <c r="C10" s="10"/>
-      <c r="D10" s="11" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="12">
         <v>10</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C11" s="14"/>
+      <c r="D11" s="15" t="s">
         <v>179</v>
-      </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="13" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="10">
         <v>11</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="16" t="s">
+        <v>180</v>
+      </c>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17" t="s">
         <v>181</v>
-      </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="11" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="12">
         <v>12</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="D13" s="15" t="s">
         <v>183</v>
-      </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="13" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="10">
         <v>13</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="16" t="s">
+        <v>184</v>
+      </c>
+      <c r="C14" s="16" t="s">
         <v>185</v>
       </c>
-      <c r="C14" s="10"/>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="17" t="s">
         <v>186</v>
       </c>
     </row>
@@ -4208,11 +4222,11 @@
       <c r="A15" s="12">
         <v>14</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="C15" s="12"/>
-      <c r="D15" s="13" t="s">
+      <c r="C15" s="14"/>
+      <c r="D15" s="15" t="s">
         <v>188</v>
       </c>
     </row>
@@ -4220,43 +4234,18 @@
       <c r="A16" s="10">
         <v>15</v>
       </c>
-      <c r="B16" s="10" t="s">
-        <v>189</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>168</v>
-      </c>
-      <c r="D16" s="11" t="s">
+      <c r="B16" s="16" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="12">
-        <v>16</v>
-      </c>
-      <c r="B17" s="12" t="s">
+      <c r="C16" s="16" t="b">
+        <v>1</v>
+      </c>
+      <c r="D16" s="17" t="s">
         <v>191</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>192</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="10">
-        <v>17</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>194</v>
-      </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="11" t="s">
-        <v>195</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fixed normalisation and added table name in diff report
</commit_message>
<xml_diff>
--- a/excel_files/analytics_dw.public.dim_vehicle_master.xlsx
+++ b/excel_files/analytics_dw.public.dim_vehicle_master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PycharmProjects\ETL_Testing_Databricks_Multi_Source\Execution\excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E115370A-859D-4C2E-8CC3-1F262005D3D6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7D8EF95-FFE2-4820-8C78-C5D956ED74F8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6936" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6936" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="mysql_server" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
changed sub path to xl_m
</commit_message>
<xml_diff>
--- a/excel_files/analytics_dw.public.dim_vehicle_master.xlsx
+++ b/excel_files/analytics_dw.public.dim_vehicle_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PycharmProjects\ETL_Testing_Databricks_Multi_Source\Execution\excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BBAFFAD-2726-413C-B256-E9F4914961BC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A988B5C0-AD72-4437-A16C-16C20CED2FDB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6936" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -607,7 +607,7 @@
     <t>analytics_dw.public.dim_vehicle_master.xlsx</t>
   </si>
   <si>
-    <t>xl</t>
+    <t>xl_m</t>
   </si>
 </sst>
 </file>

</xml_diff>